<commit_message>
BIS-2726: Fixed Type Group export in AdminUI, improvements to type group import
</commit_message>
<xml_diff>
--- a/server-application-server/sourceTest/java/ch/ethz/sis/openbis/generic/server/xls/export/resources/export-sample-type-internal.xlsx
+++ b/server-application-server/sourceTest/java/ch/ethz/sis/openbis/generic/server/xls/export/resources/export-sample-type-internal.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="54">
   <si>
     <t xml:space="preserve">TYPE_GROUP</t>
   </si>
@@ -55,12 +55,15 @@
     <t xml:space="preserve">2023-03-11 17:23:44</t>
   </si>
   <si>
+    <t xml:space="preserve">INTERNAL_ENTRY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FALSE</t>
+  </si>
+  <si>
     <t xml:space="preserve">TEST_GROUP_1</t>
   </si>
   <si>
-    <t xml:space="preserve">FALSE</t>
-  </si>
-  <si>
     <t xml:space="preserve">SAMPLE_TYPE</t>
   </si>
   <si>
@@ -92,9 +95,6 @@
   </si>
   <si>
     <t xml:space="preserve">Meta Data</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INTERNAL_ENTRY</t>
   </si>
   <si>
     <t xml:space="preserve">Internal Entry</t>
@@ -350,8 +350,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:S15"/>
-  <sheetFormatPr defaultColWidth="10.859375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:S19"/>
+  <sheetFormatPr defaultColWidth="10.8671875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="21.95"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="15.28"/>
@@ -397,54 +397,73 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="5" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="2"/>
-    </row>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="C7" s="2"/>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B8" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C8" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D8" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E8" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F8" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="0" t="s">
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="0" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>10</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4"/>
-      <c r="D8" s="2"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -455,260 +474,297 @@
         <v>2</v>
       </c>
       <c r="C10" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4"/>
+      <c r="D12" s="2"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="3" t="s">
+    </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="D14" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="E14" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="G10" s="3" t="s">
+      <c r="F14" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="H10" s="3" t="s">
+      <c r="G14" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H14" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="I10" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="J10" s="3" t="s">
+      <c r="I14" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="K10" s="3" t="s">
+      <c r="J14" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="L10" s="3" t="s">
+      <c r="K14" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="M10" s="6" t="s">
+      <c r="L14" s="3" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+      <c r="M14" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11" s="2" t="s">
+    </row>
+    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E11" s="2" t="s">
+      <c r="D15" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="F15" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="G11" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="H11" s="2" t="s">
+      <c r="G15" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H15" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2"/>
-      <c r="K11" s="2"/>
-      <c r="L11" s="7" t="s">
+      <c r="I15" s="2"/>
+      <c r="J15" s="2"/>
+      <c r="K15" s="2"/>
+      <c r="L15" s="7" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B16" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C16" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D16" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="E16" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="F16" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="G12" s="3" t="s">
+      <c r="G16" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="H12" s="3" t="s">
+      <c r="H16" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="I12" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="J12" s="3" t="s">
+      <c r="I16" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="J16" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="K12" s="3" t="s">
+      <c r="K16" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="L12" s="3" t="s">
+      <c r="L16" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="M12" s="3" t="s">
+      <c r="M16" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="N12" s="3" t="s">
+      <c r="N16" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="O12" s="3" t="s">
+      <c r="O16" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="P12" s="3" t="s">
+      <c r="P16" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="Q12" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="R12" s="3" t="s">
+      <c r="Q16" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="S12" s="3" t="s">
+      <c r="R16" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
+      <c r="S16" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E13" s="2" t="s">
+      <c r="B17" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E17" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="F17" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="G13" s="2" t="s">
+      <c r="G17" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2" t="s">
+      <c r="H17" s="2"/>
+      <c r="I17" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
-      <c r="L13" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M13" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N13" s="2"/>
-      <c r="O13" s="2"/>
-      <c r="P13" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="Q13" s="2"/>
-      <c r="R13" s="2"/>
-      <c r="S13" s="2"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+      <c r="J17" s="2"/>
+      <c r="K17" s="2"/>
+      <c r="L17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N17" s="2"/>
+      <c r="O17" s="2"/>
+      <c r="P17" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="Q17" s="2"/>
+      <c r="R17" s="2"/>
+      <c r="S17" s="2"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E14" s="2" t="s">
+      <c r="B18" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E18" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="F18" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="G14" s="2" t="s">
+      <c r="G18" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2" t="s">
+      <c r="H18" s="2"/>
+      <c r="I18" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="J14" s="2" t="s">
+      <c r="J18" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="K14" s="2"/>
-      <c r="L14" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M14" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N14" s="2"/>
-      <c r="O14" s="2"/>
-      <c r="P14" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q14" s="2"/>
-      <c r="R14" s="2"/>
-      <c r="S14" s="2"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
+      <c r="K18" s="2"/>
+      <c r="L18" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M18" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N18" s="2"/>
+      <c r="O18" s="2"/>
+      <c r="P18" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q18" s="2"/>
+      <c r="R18" s="2"/>
+      <c r="S18" s="2"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2" t="s">
+      <c r="B19" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="G19" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2" t="s">
+      <c r="H19" s="2"/>
+      <c r="I19" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="J15" s="2"/>
-      <c r="K15" s="2" t="s">
+      <c r="J19" s="2"/>
+      <c r="K19" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="L15" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M15" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N15" s="2"/>
-      <c r="O15" s="2"/>
-      <c r="P15" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q15" s="2"/>
-      <c r="R15" s="2"/>
-      <c r="S15" s="2"/>
+      <c r="L19" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M19" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N19" s="2"/>
+      <c r="O19" s="2"/>
+      <c r="P19" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q19" s="2"/>
+      <c r="R19" s="2"/>
+      <c r="S19" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>